<commit_message>
ejercicio 9 de secuenciales
</commit_message>
<xml_diff>
--- a/Varios/Relacion entre ejercicios guia vs web.xlsx
+++ b/Varios/Relacion entre ejercicios guia vs web.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\2026_AED\_Guia_Ejercicios\0_Varios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\2026_AED\AED26_Guia_Ejercicios\Varios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978B73CF-EE63-47A3-A1D6-2017CD00C1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69BC7A15-7A77-4831-8A69-70F67332D8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="16245" windowHeight="13755" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="285">
   <si>
     <t>1.1.5.1</t>
   </si>
@@ -891,22 +891,17 @@
   </si>
   <si>
     <t>3.32</t>
+  </si>
+  <si>
+    <t>complejo para iniciar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -960,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -974,9 +969,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -986,7 +978,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1330,7 +1328,7 @@
     <col min="1" max="1" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.7109375" style="1" customWidth="1"/>
     <col min="3" max="5" width="9.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
@@ -1350,7 +1348,7 @@
       <c r="E1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="8" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1429,16 +1427,16 @@
       <c r="B6" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>5</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="7">
-        <v>0</v>
-      </c>
-      <c r="F6" s="6"/>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1456,6 +1454,7 @@
       <c r="E7" s="1">
         <v>1</v>
       </c>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1473,6 +1472,7 @@
       <c r="E8" s="1">
         <v>1</v>
       </c>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1507,6 +1507,7 @@
       <c r="E10" s="1">
         <v>1</v>
       </c>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1524,6 +1525,7 @@
       <c r="E11" s="1">
         <v>1</v>
       </c>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1541,6 +1543,7 @@
       <c r="E12" s="1">
         <v>1</v>
       </c>
+      <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1558,6 +1561,7 @@
       <c r="E13" s="1">
         <v>1</v>
       </c>
+      <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1592,6 +1596,7 @@
       <c r="E15" s="1">
         <v>1</v>
       </c>
+      <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
@@ -1609,11 +1614,11 @@
       <c r="E16" s="3">
         <v>1</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -1627,11 +1632,13 @@
         <v>21</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1</v>
       </c>
@@ -1645,7 +1652,7 @@
         <v>22</v>
       </c>
       <c r="E18" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1766,7 +1773,7 @@
       <c r="E25" s="3">
         <v>0</v>
       </c>
-      <c r="F25" s="6"/>
+      <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -2039,7 +2046,6 @@
       <c r="E41" s="1">
         <v>0</v>
       </c>
-      <c r="F41" s="5"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
@@ -2159,7 +2165,7 @@
       <c r="E48" s="3">
         <v>0</v>
       </c>
-      <c r="F48" s="6"/>
+      <c r="F48" s="9"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
@@ -2364,7 +2370,7 @@
       <c r="E60" s="3">
         <v>0</v>
       </c>
-      <c r="F60" s="6"/>
+      <c r="F60" s="9"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
@@ -2478,7 +2484,7 @@
       <c r="E68" s="3">
         <v>0</v>
       </c>
-      <c r="F68" s="6"/>
+      <c r="F68" s="9"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
@@ -3023,7 +3029,7 @@
       <c r="E100" s="3">
         <v>0</v>
       </c>
-      <c r="F100" s="6"/>
+      <c r="F100" s="9"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
@@ -3092,7 +3098,7 @@
       <c r="E104" s="3">
         <v>0</v>
       </c>
-      <c r="F104" s="6"/>
+      <c r="F104" s="9"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
@@ -3246,7 +3252,7 @@
       <c r="E113" s="3">
         <v>0</v>
       </c>
-      <c r="F113" s="6"/>
+      <c r="F113" s="9"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
@@ -3349,7 +3355,7 @@
       <c r="E119" s="3">
         <v>0</v>
       </c>
-      <c r="F119" s="6"/>
+      <c r="F119" s="9"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
@@ -3401,7 +3407,7 @@
       <c r="E122" s="3">
         <v>0</v>
       </c>
-      <c r="F122" s="6"/>
+      <c r="F122" s="9"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
@@ -3521,7 +3527,7 @@
       <c r="E129" s="3">
         <v>0</v>
       </c>
-      <c r="F129" s="6"/>
+      <c r="F129" s="9"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
@@ -3590,7 +3596,7 @@
       <c r="E133" s="1">
         <v>0</v>
       </c>
-      <c r="F133" s="4" t="s">
+      <c r="F133" s="8" t="s">
         <v>241</v>
       </c>
     </row>
@@ -3627,7 +3633,7 @@
       <c r="E135" s="1">
         <v>0</v>
       </c>
-      <c r="F135" s="4" t="s">
+      <c r="F135" s="8" t="s">
         <v>244</v>
       </c>
     </row>
@@ -3732,7 +3738,7 @@
       <c r="E141" s="3">
         <v>0</v>
       </c>
-      <c r="F141" s="6"/>
+      <c r="F141" s="9"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
@@ -3902,7 +3908,7 @@
       <c r="E153" s="3">
         <v>0</v>
       </c>
-      <c r="F153" s="6"/>
+      <c r="F153" s="9"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
@@ -3974,7 +3980,7 @@
       <c r="E158" s="3">
         <v>0</v>
       </c>
-      <c r="F158" s="6"/>
+      <c r="F158" s="9"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
@@ -4032,7 +4038,7 @@
       <c r="E162" s="3">
         <v>0</v>
       </c>
-      <c r="F162" s="6"/>
+      <c r="F162" s="9"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
@@ -4146,23 +4152,23 @@
       <c r="E170" s="3">
         <v>0</v>
       </c>
-      <c r="F170" s="6"/>
+      <c r="F170" s="9"/>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A171" s="8" t="s">
+      <c r="A171" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B171" s="8" t="s">
+      <c r="B171" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="C171" s="8">
-        <v>1</v>
-      </c>
-      <c r="D171" s="8"/>
-      <c r="E171" s="8">
-        <v>0</v>
-      </c>
-      <c r="F171" s="9"/>
+      <c r="C171" s="7">
+        <v>1</v>
+      </c>
+      <c r="D171" s="7"/>
+      <c r="E171" s="7">
+        <v>0</v>
+      </c>
+      <c r="F171" s="10"/>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
@@ -4178,7 +4184,7 @@
       <c r="E172" s="3">
         <v>0</v>
       </c>
-      <c r="F172" s="6"/>
+      <c r="F172" s="9"/>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
@@ -4417,7 +4423,7 @@
       <c r="E186" s="1">
         <v>0</v>
       </c>
-      <c r="F186" s="4" t="s">
+      <c r="F186" s="8" t="s">
         <v>265</v>
       </c>
     </row>
@@ -4726,7 +4732,7 @@
       <c r="E204" s="3">
         <v>0</v>
       </c>
-      <c r="F204" s="6"/>
+      <c r="F204" s="9"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
@@ -4840,7 +4846,7 @@
       <c r="E212" s="3">
         <v>0</v>
       </c>
-      <c r="F212" s="6"/>
+      <c r="F212" s="9"/>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
@@ -5080,7 +5086,7 @@
       <c r="E229" s="3">
         <v>0</v>
       </c>
-      <c r="F229" s="6"/>
+      <c r="F229" s="9"/>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
@@ -5208,7 +5214,7 @@
       <c r="E238" s="3">
         <v>0</v>
       </c>
-      <c r="F238" s="6"/>
+      <c r="F238" s="9"/>
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
@@ -5378,7 +5384,7 @@
       <c r="E250" s="3">
         <v>0</v>
       </c>
-      <c r="F250" s="6"/>
+      <c r="F250" s="9"/>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
@@ -5562,7 +5568,7 @@
       <c r="E263" s="3">
         <v>0</v>
       </c>
-      <c r="F263" s="6"/>
+      <c r="F263" s="9"/>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
@@ -5620,23 +5626,23 @@
       <c r="E267" s="3">
         <v>0</v>
       </c>
-      <c r="F267" s="6"/>
+      <c r="F267" s="9"/>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A268" s="8">
+      <c r="A268" s="7">
         <v>6</v>
       </c>
-      <c r="B268" s="8" t="s">
+      <c r="B268" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="C268" s="8">
-        <v>1</v>
-      </c>
-      <c r="D268" s="8"/>
-      <c r="E268" s="8">
-        <v>0</v>
-      </c>
-      <c r="F268" s="9"/>
+      <c r="C268" s="7">
+        <v>1</v>
+      </c>
+      <c r="D268" s="7"/>
+      <c r="E268" s="7">
+        <v>0</v>
+      </c>
+      <c r="F268" s="10"/>
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
@@ -5709,20 +5715,20 @@
       </c>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A274" s="8" t="s">
+      <c r="A274" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B274" s="8" t="s">
+      <c r="B274" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C274" s="8">
+      <c r="C274" s="7">
         <v>6</v>
       </c>
-      <c r="D274" s="8"/>
-      <c r="E274" s="8">
-        <v>0</v>
-      </c>
-      <c r="F274" s="9"/>
+      <c r="D274" s="7"/>
+      <c r="E274" s="7">
+        <v>0</v>
+      </c>
+      <c r="F274" s="10"/>
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
@@ -5794,7 +5800,7 @@
       <c r="E279" s="3">
         <v>0</v>
       </c>
-      <c r="F279" s="6"/>
+      <c r="F279" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F279" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}">
@@ -5804,7 +5810,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="iconSet" priority="1">
       <iconSet>

</xml_diff>

<commit_message>
Desarrollo ejercicio 14 compra supermercado
</commit_message>
<xml_diff>
--- a/Varios/Relacion entre ejercicios guia vs web.xlsx
+++ b/Varios/Relacion entre ejercicios guia vs web.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\2026_AED\AED26_Guia_Ejercicios\Varios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42FA6B3D-8E23-41BE-9D57-4ACD5C7B2D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8917D7BD-0FA9-4324-BC1F-EF46D51FB9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
+    <workbookView xWindow="13275" yWindow="1095" windowWidth="14790" windowHeight="14070" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1315,7 +1315,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F279"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1432,7 +1431,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -1449,7 +1448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -1480,10 +1479,10 @@
         <v>9</v>
       </c>
       <c r="E9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -1500,7 +1499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -1517,7 +1516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -1534,7 +1533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -1565,10 +1564,10 @@
         <v>15</v>
       </c>
       <c r="E14" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>1</v>
       </c>
@@ -1585,7 +1584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>1</v>
       </c>
@@ -1605,7 +1604,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -1625,7 +1624,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1</v>
       </c>
@@ -1642,7 +1641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -1659,7 +1658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1676,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>1</v>
       </c>
@@ -1707,7 +1706,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1741,7 +1740,7 @@
         <v>28</v>
       </c>
       <c r="E24" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1758,7 +1757,7 @@
         <v>7</v>
       </c>
       <c r="E25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5"/>
     </row>
@@ -5790,13 +5789,7 @@
       <c r="F279" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F279" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="0"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F279" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="iconSet" priority="1">

</xml_diff>

<commit_message>
cambios menores archivo de relacion de ejercicios
</commit_message>
<xml_diff>
--- a/Varios/Relacion entre ejercicios guia vs web.xlsx
+++ b/Varios/Relacion entre ejercicios guia vs web.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\2026_AED\AED26_Guia_Ejercicios\Varios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8917D7BD-0FA9-4324-BC1F-EF46D51FB9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A23ECDD-486A-49C2-AA0C-FF4D374D53DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13275" yWindow="1095" windowWidth="14790" windowHeight="14070" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
+    <workbookView xWindow="11700" yWindow="855" windowWidth="14790" windowHeight="14070" xr2:uid="{B06F9037-2334-4A9B-96A2-685548E21E24}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$278</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="285">
   <si>
     <t>1.1.5.1</t>
   </si>
@@ -1315,7 +1315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}">
-  <dimension ref="A1:F279"/>
+  <dimension ref="A1:F278"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1754,7 +1754,7 @@
         <v>14</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E25" s="3">
         <v>1</v>
@@ -1768,11 +1768,11 @@
       <c r="B26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>31</v>
+      <c r="C26" s="1">
+        <v>15</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
@@ -1786,10 +1786,10 @@
         <v>32</v>
       </c>
       <c r="C27" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E27" s="1">
         <v>0</v>
@@ -1803,10 +1803,10 @@
         <v>32</v>
       </c>
       <c r="C28" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E28" s="1">
         <v>0</v>
@@ -1820,10 +1820,10 @@
         <v>32</v>
       </c>
       <c r="C29" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E29" s="1">
         <v>0</v>
@@ -1837,10 +1837,10 @@
         <v>32</v>
       </c>
       <c r="C30" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
@@ -1853,11 +1853,11 @@
       <c r="B31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="1">
-        <v>19</v>
+      <c r="C31" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E31" s="1">
         <v>0</v>
@@ -1874,7 +1874,7 @@
         <v>31</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E32" s="1">
         <v>0</v>
@@ -1891,7 +1891,7 @@
         <v>31</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E33" s="1">
         <v>0</v>
@@ -1904,11 +1904,11 @@
       <c r="B34" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>31</v>
+      <c r="C34" s="1">
+        <v>20</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E34" s="1">
         <v>0</v>
@@ -1922,10 +1922,10 @@
         <v>32</v>
       </c>
       <c r="C35" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E35" s="1">
         <v>0</v>
@@ -1939,10 +1939,10 @@
         <v>32</v>
       </c>
       <c r="C36" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E36" s="1">
         <v>0</v>
@@ -1956,10 +1956,10 @@
         <v>32</v>
       </c>
       <c r="C37" s="1">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E37" s="1">
         <v>0</v>
@@ -1972,11 +1972,11 @@
       <c r="B38" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C38" s="1">
-        <v>23</v>
+      <c r="C38" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
@@ -1993,7 +1993,7 @@
         <v>31</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E39" s="1">
         <v>0</v>
@@ -2006,11 +2006,11 @@
       <c r="B40" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>31</v>
+      <c r="C40" s="1">
+        <v>24</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E40" s="1">
         <v>0</v>
@@ -2024,10 +2024,10 @@
         <v>32</v>
       </c>
       <c r="C41" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E41" s="1">
         <v>0</v>
@@ -2041,10 +2041,10 @@
         <v>32</v>
       </c>
       <c r="C42" s="1">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E42" s="1">
         <v>0</v>
@@ -2058,10 +2058,10 @@
         <v>32</v>
       </c>
       <c r="C43" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E43" s="1">
         <v>0</v>
@@ -2075,10 +2075,10 @@
         <v>32</v>
       </c>
       <c r="C44" s="1">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E44" s="1">
         <v>0</v>
@@ -2092,10 +2092,10 @@
         <v>32</v>
       </c>
       <c r="C45" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E45" s="1">
         <v>0</v>
@@ -2109,49 +2109,49 @@
         <v>32</v>
       </c>
       <c r="C46" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E46" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
-        <v>1</v>
-      </c>
-      <c r="B47" s="1" t="s">
+      <c r="A47" s="3">
+        <v>1</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C47" s="1">
-        <v>30</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E47" s="1">
-        <v>0</v>
-      </c>
+      <c r="C47" s="3">
+        <v>31</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E47" s="3">
+        <v>0</v>
+      </c>
+      <c r="F47" s="5"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="3">
-        <v>1</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C48" s="3">
-        <v>31</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E48" s="3">
-        <v>0</v>
-      </c>
-      <c r="F48" s="5"/>
+      <c r="A48" s="1">
+        <v>1</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E48" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
@@ -2161,10 +2161,10 @@
         <v>65</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E49" s="1">
         <v>0</v>
@@ -2178,10 +2178,10 @@
         <v>65</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E50" s="1">
         <v>0</v>
@@ -2195,10 +2195,10 @@
         <v>65</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E51" s="1">
         <v>0</v>
@@ -2212,10 +2212,10 @@
         <v>65</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E52" s="1">
         <v>0</v>
@@ -2229,10 +2229,10 @@
         <v>65</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E53" s="1">
         <v>0</v>
@@ -2246,10 +2246,10 @@
         <v>65</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E54" s="1">
         <v>0</v>
@@ -2263,10 +2263,10 @@
         <v>65</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E55" s="1">
         <v>0</v>
@@ -2280,10 +2280,10 @@
         <v>65</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E56" s="1">
         <v>0</v>
@@ -2297,10 +2297,10 @@
         <v>65</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E57" s="1">
         <v>0</v>
@@ -2314,49 +2314,46 @@
         <v>65</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E58" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
-        <v>1</v>
-      </c>
-      <c r="B59" s="1" t="s">
+      <c r="A59" s="3">
+        <v>1</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="E59" s="1">
-        <v>0</v>
-      </c>
+      <c r="C59" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E59" s="3">
+        <v>0</v>
+      </c>
+      <c r="F59" s="5"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="3">
-        <v>1</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="E60" s="3">
-        <v>0</v>
-      </c>
-      <c r="F60" s="5"/>
+      <c r="A60" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" s="1">
+        <v>1</v>
+      </c>
+      <c r="E60" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
@@ -2366,7 +2363,7 @@
         <v>79</v>
       </c>
       <c r="C61" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="1">
         <v>0</v>
@@ -2380,7 +2377,7 @@
         <v>79</v>
       </c>
       <c r="C62" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62" s="1">
         <v>0</v>
@@ -2394,7 +2391,7 @@
         <v>79</v>
       </c>
       <c r="C63" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E63" s="1">
         <v>0</v>
@@ -2408,7 +2405,7 @@
         <v>79</v>
       </c>
       <c r="C64" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E64" s="1">
         <v>0</v>
@@ -2422,7 +2419,7 @@
         <v>79</v>
       </c>
       <c r="C65" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1">
         <v>0</v>
@@ -2436,41 +2433,44 @@
         <v>79</v>
       </c>
       <c r="C66" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
+      <c r="A67" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C67" s="1">
-        <v>7</v>
-      </c>
-      <c r="E67" s="1">
-        <v>0</v>
-      </c>
+      <c r="C67" s="3">
+        <v>8</v>
+      </c>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3">
+        <v>0</v>
+      </c>
+      <c r="F67" s="5"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C68" s="3">
-        <v>8</v>
-      </c>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3">
-        <v>0</v>
-      </c>
-      <c r="F68" s="5"/>
+      <c r="A68" s="1">
+        <v>2</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E68" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
@@ -2480,10 +2480,10 @@
         <v>80</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E69" s="1">
         <v>0</v>
@@ -2497,10 +2497,10 @@
         <v>80</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E70" s="1">
         <v>0</v>
@@ -2514,10 +2514,10 @@
         <v>80</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E71" s="1">
         <v>0</v>
@@ -2531,10 +2531,10 @@
         <v>80</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E72" s="1">
         <v>0</v>
@@ -2548,10 +2548,10 @@
         <v>80</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E73" s="1">
         <v>0</v>
@@ -2565,10 +2565,10 @@
         <v>80</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E74" s="1">
         <v>0</v>
@@ -2582,10 +2582,10 @@
         <v>80</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E75" s="1">
         <v>0</v>
@@ -2599,10 +2599,10 @@
         <v>80</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E76" s="1">
         <v>0</v>
@@ -2616,10 +2616,10 @@
         <v>80</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E77" s="1">
         <v>0</v>
@@ -2633,10 +2633,10 @@
         <v>80</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E78" s="1">
         <v>0</v>
@@ -2650,10 +2650,10 @@
         <v>80</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E79" s="1">
         <v>0</v>
@@ -2667,10 +2667,10 @@
         <v>80</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E80" s="1">
         <v>0</v>
@@ -2684,10 +2684,10 @@
         <v>80</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E81" s="1">
         <v>0</v>
@@ -2701,10 +2701,10 @@
         <v>80</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E82" s="1">
         <v>0</v>
@@ -2718,10 +2718,10 @@
         <v>80</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E83" s="1">
         <v>0</v>
@@ -2735,10 +2735,10 @@
         <v>80</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E84" s="1">
         <v>0</v>
@@ -2752,10 +2752,10 @@
         <v>80</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E85" s="1">
         <v>0</v>
@@ -2769,10 +2769,10 @@
         <v>80</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E86" s="1">
         <v>0</v>
@@ -2786,10 +2786,10 @@
         <v>80</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E87" s="1">
         <v>0</v>
@@ -2803,10 +2803,10 @@
         <v>80</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E88" s="1">
         <v>0</v>
@@ -2820,10 +2820,10 @@
         <v>80</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E89" s="1">
         <v>0</v>
@@ -2837,10 +2837,10 @@
         <v>80</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E90" s="1">
         <v>0</v>
@@ -2854,10 +2854,10 @@
         <v>80</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E91" s="1">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>80</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E92" s="1">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>80</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E93" s="1">
         <v>0</v>
@@ -2905,10 +2905,10 @@
         <v>80</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E94" s="1">
         <v>0</v>
@@ -2922,10 +2922,10 @@
         <v>80</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E95" s="1">
         <v>0</v>
@@ -2939,10 +2939,10 @@
         <v>80</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>108</v>
+        <v>7</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E96" s="1">
         <v>0</v>
@@ -2959,7 +2959,7 @@
         <v>7</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E97" s="1">
         <v>0</v>
@@ -2976,46 +2976,46 @@
         <v>7</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E98" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="1">
-        <v>2</v>
-      </c>
-      <c r="B99" s="1" t="s">
+      <c r="A99" s="3">
+        <v>2</v>
+      </c>
+      <c r="B99" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C99" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D99" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="E99" s="1">
-        <v>0</v>
-      </c>
+      <c r="D99" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E99" s="3">
+        <v>0</v>
+      </c>
+      <c r="F99" s="5"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="3">
-        <v>2</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C100" s="3" t="s">
+      <c r="A100" s="1">
+        <v>2</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D100" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E100" s="3">
-        <v>0</v>
-      </c>
-      <c r="F100" s="5"/>
+      <c r="D100" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E100" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
@@ -3028,7 +3028,7 @@
         <v>7</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E101" s="1">
         <v>0</v>
@@ -3045,46 +3045,46 @@
         <v>7</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="E102" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" s="1">
-        <v>2</v>
-      </c>
-      <c r="B103" s="1" t="s">
+      <c r="A103" s="3">
+        <v>2</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="C103" s="1" t="s">
+      <c r="C103" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D103" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="E103" s="1">
-        <v>0</v>
-      </c>
+      <c r="D103" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E103" s="3">
+        <v>0</v>
+      </c>
+      <c r="F103" s="5"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A104" s="3">
-        <v>2</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C104" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D104" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E104" s="3">
-        <v>0</v>
-      </c>
-      <c r="F104" s="5"/>
+      <c r="A104" s="1">
+        <v>2</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E104" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
@@ -3094,10 +3094,10 @@
         <v>109</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E105" s="1">
         <v>0</v>
@@ -3111,10 +3111,10 @@
         <v>109</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E106" s="1">
         <v>0</v>
@@ -3128,10 +3128,10 @@
         <v>109</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E107" s="1">
         <v>0</v>
@@ -3145,10 +3145,10 @@
         <v>109</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E108" s="1">
         <v>0</v>
@@ -3162,10 +3162,10 @@
         <v>109</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E109" s="1">
         <v>0</v>
@@ -3179,10 +3179,10 @@
         <v>109</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E110" s="1">
         <v>0</v>
@@ -3196,49 +3196,49 @@
         <v>109</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E111" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="1">
-        <v>2</v>
-      </c>
-      <c r="B112" s="1" t="s">
+      <c r="A112" s="3">
+        <v>2</v>
+      </c>
+      <c r="B112" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C112" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="D112" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="E112" s="1">
-        <v>0</v>
-      </c>
+      <c r="C112" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E112" s="3">
+        <v>0</v>
+      </c>
+      <c r="F112" s="5"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" s="3">
-        <v>2</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D113" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E113" s="3">
-        <v>0</v>
-      </c>
-      <c r="F113" s="5"/>
+      <c r="A113" s="1">
+        <v>2</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E113" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
@@ -3248,10 +3248,10 @@
         <v>119</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E114" s="1">
         <v>0</v>
@@ -3265,10 +3265,10 @@
         <v>119</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E115" s="1">
         <v>0</v>
@@ -3282,10 +3282,10 @@
         <v>119</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E116" s="1">
         <v>0</v>
@@ -3299,49 +3299,49 @@
         <v>119</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E117" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A118" s="1">
-        <v>2</v>
-      </c>
-      <c r="B118" s="1" t="s">
+      <c r="A118" s="3">
+        <v>2</v>
+      </c>
+      <c r="B118" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C118" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D118" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="E118" s="1">
-        <v>0</v>
-      </c>
+      <c r="C118" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E118" s="3">
+        <v>0</v>
+      </c>
+      <c r="F118" s="5"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A119" s="3">
-        <v>2</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E119" s="3">
-        <v>0</v>
-      </c>
-      <c r="F119" s="5"/>
+      <c r="A119" s="1">
+        <v>2</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E119" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
@@ -3351,49 +3351,49 @@
         <v>126</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E120" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A121" s="1">
-        <v>2</v>
-      </c>
-      <c r="B121" s="1" t="s">
+      <c r="A121" s="3">
+        <v>2</v>
+      </c>
+      <c r="B121" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C121" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="E121" s="1">
-        <v>0</v>
-      </c>
+      <c r="C121" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E121" s="3">
+        <v>0</v>
+      </c>
+      <c r="F121" s="5"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" s="3">
-        <v>2</v>
-      </c>
-      <c r="B122" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="E122" s="3">
-        <v>0</v>
-      </c>
-      <c r="F122" s="5"/>
+      <c r="A122" s="1">
+        <v>2</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="E122" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
@@ -3403,10 +3403,10 @@
         <v>130</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E123" s="1">
         <v>0</v>
@@ -3420,10 +3420,10 @@
         <v>130</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E124" s="1">
         <v>0</v>
@@ -3437,10 +3437,10 @@
         <v>130</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E125" s="1">
         <v>0</v>
@@ -3454,10 +3454,10 @@
         <v>130</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E126" s="1">
         <v>0</v>
@@ -3471,49 +3471,49 @@
         <v>130</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E127" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128" s="1">
-        <v>2</v>
-      </c>
-      <c r="B128" s="1" t="s">
+      <c r="A128" s="3">
+        <v>2</v>
+      </c>
+      <c r="B128" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C128" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="E128" s="1">
-        <v>0</v>
-      </c>
+      <c r="C128" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E128" s="3">
+        <v>0</v>
+      </c>
+      <c r="F128" s="5"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129" s="3">
-        <v>2</v>
-      </c>
-      <c r="B129" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D129" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E129" s="3">
-        <v>0</v>
-      </c>
-      <c r="F129" s="5"/>
+      <c r="A129" s="1">
+        <v>2</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="E129" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
@@ -3523,10 +3523,10 @@
         <v>138</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>7</v>
+        <v>139</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E130" s="1">
         <v>0</v>
@@ -3540,10 +3540,10 @@
         <v>138</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E131" s="1">
         <v>0</v>
@@ -3557,13 +3557,16 @@
         <v>138</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E132" s="1">
         <v>0</v>
+      </c>
+      <c r="F132" s="4" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -3574,16 +3577,13 @@
         <v>138</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E133" s="1">
         <v>0</v>
-      </c>
-      <c r="F133" s="4" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -3594,13 +3594,16 @@
         <v>138</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E134" s="1">
         <v>0</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -3611,16 +3614,13 @@
         <v>138</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E135" s="1">
         <v>0</v>
-      </c>
-      <c r="F135" s="4" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -3631,10 +3631,10 @@
         <v>138</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E136" s="1">
         <v>0</v>
@@ -3648,10 +3648,10 @@
         <v>138</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E137" s="1">
         <v>0</v>
@@ -3665,10 +3665,10 @@
         <v>138</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E138" s="1">
         <v>0</v>
@@ -3682,49 +3682,46 @@
         <v>138</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>147</v>
+        <v>7</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E139" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A140" s="1">
-        <v>2</v>
-      </c>
-      <c r="B140" s="1" t="s">
+      <c r="A140" s="3">
+        <v>2</v>
+      </c>
+      <c r="B140" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C140" s="1" t="s">
+      <c r="C140" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D140" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="E140" s="1">
-        <v>0</v>
-      </c>
+      <c r="D140" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E140" s="3">
+        <v>0</v>
+      </c>
+      <c r="F140" s="5"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A141" s="3">
-        <v>2</v>
-      </c>
-      <c r="B141" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C141" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D141" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="E141" s="3">
-        <v>0</v>
-      </c>
-      <c r="F141" s="5"/>
+      <c r="A141" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C141" s="1">
+        <v>1</v>
+      </c>
+      <c r="E141" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
@@ -3734,7 +3731,7 @@
         <v>149</v>
       </c>
       <c r="C142" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" s="1">
         <v>0</v>
@@ -3748,7 +3745,7 @@
         <v>149</v>
       </c>
       <c r="C143" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E143" s="1">
         <v>0</v>
@@ -3762,7 +3759,7 @@
         <v>149</v>
       </c>
       <c r="C144" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E144" s="1">
         <v>0</v>
@@ -3776,7 +3773,7 @@
         <v>149</v>
       </c>
       <c r="C145" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E145" s="1">
         <v>0</v>
@@ -3790,7 +3787,7 @@
         <v>149</v>
       </c>
       <c r="C146" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E146" s="1">
         <v>0</v>
@@ -3804,7 +3801,7 @@
         <v>149</v>
       </c>
       <c r="C147" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E147" s="1">
         <v>0</v>
@@ -3818,7 +3815,7 @@
         <v>149</v>
       </c>
       <c r="C148" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E148" s="1">
         <v>0</v>
@@ -3832,7 +3829,7 @@
         <v>149</v>
       </c>
       <c r="C149" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E149" s="1">
         <v>0</v>
@@ -3846,7 +3843,7 @@
         <v>149</v>
       </c>
       <c r="C150" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E150" s="1">
         <v>0</v>
@@ -3860,41 +3857,41 @@
         <v>149</v>
       </c>
       <c r="C151" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E151" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A152" s="1" t="s">
+      <c r="A152" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B152" s="1" t="s">
+      <c r="B152" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C152" s="1">
-        <v>11</v>
-      </c>
-      <c r="E152" s="1">
-        <v>0</v>
-      </c>
+      <c r="C152" s="3">
+        <v>12</v>
+      </c>
+      <c r="D152" s="3"/>
+      <c r="E152" s="3">
+        <v>0</v>
+      </c>
+      <c r="F152" s="5"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A153" s="3" t="s">
+      <c r="A153" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B153" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C153" s="3">
-        <v>12</v>
-      </c>
-      <c r="D153" s="3"/>
-      <c r="E153" s="3">
-        <v>0</v>
-      </c>
-      <c r="F153" s="5"/>
+      <c r="B153" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C153" s="1">
+        <v>1</v>
+      </c>
+      <c r="E153" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
@@ -3904,7 +3901,7 @@
         <v>150</v>
       </c>
       <c r="C154" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="1">
         <v>0</v>
@@ -3918,7 +3915,7 @@
         <v>150</v>
       </c>
       <c r="C155" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E155" s="1">
         <v>0</v>
@@ -3932,41 +3929,41 @@
         <v>150</v>
       </c>
       <c r="C156" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E156" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A157" s="1" t="s">
+      <c r="A157" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B157" s="1" t="s">
+      <c r="B157" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C157" s="1">
-        <v>4</v>
-      </c>
-      <c r="E157" s="1">
-        <v>0</v>
-      </c>
+      <c r="C157" s="3">
+        <v>5</v>
+      </c>
+      <c r="D157" s="3"/>
+      <c r="E157" s="3">
+        <v>0</v>
+      </c>
+      <c r="F157" s="5"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A158" s="3" t="s">
+      <c r="A158" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B158" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C158" s="3">
-        <v>5</v>
-      </c>
-      <c r="D158" s="3"/>
-      <c r="E158" s="3">
-        <v>0</v>
-      </c>
-      <c r="F158" s="5"/>
+      <c r="B158" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C158" s="1">
+        <v>6</v>
+      </c>
+      <c r="E158" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
@@ -3976,7 +3973,7 @@
         <v>151</v>
       </c>
       <c r="C159" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E159" s="1">
         <v>0</v>
@@ -3990,41 +3987,41 @@
         <v>151</v>
       </c>
       <c r="C160" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E160" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A161" s="1" t="s">
+      <c r="A161" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B161" s="1" t="s">
+      <c r="B161" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C161" s="1">
-        <v>8</v>
-      </c>
-      <c r="E161" s="1">
-        <v>0</v>
-      </c>
+      <c r="C161" s="3">
+        <v>9</v>
+      </c>
+      <c r="D161" s="3"/>
+      <c r="E161" s="3">
+        <v>0</v>
+      </c>
+      <c r="F161" s="5"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A162" s="3" t="s">
+      <c r="A162" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B162" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C162" s="3">
-        <v>9</v>
-      </c>
-      <c r="D162" s="3"/>
-      <c r="E162" s="3">
-        <v>0</v>
-      </c>
-      <c r="F162" s="5"/>
+      <c r="B162" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C162" s="1">
+        <v>10</v>
+      </c>
+      <c r="E162" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
@@ -4034,7 +4031,7 @@
         <v>152</v>
       </c>
       <c r="C163" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E163" s="1">
         <v>0</v>
@@ -4048,7 +4045,7 @@
         <v>152</v>
       </c>
       <c r="C164" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E164" s="1">
         <v>0</v>
@@ -4062,7 +4059,7 @@
         <v>152</v>
       </c>
       <c r="C165" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E165" s="1">
         <v>0</v>
@@ -4076,7 +4073,7 @@
         <v>152</v>
       </c>
       <c r="C166" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E166" s="1">
         <v>0</v>
@@ -4090,7 +4087,7 @@
         <v>152</v>
       </c>
       <c r="C167" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E167" s="1">
         <v>0</v>
@@ -4104,73 +4101,76 @@
         <v>152</v>
       </c>
       <c r="C168" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E168" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A169" s="1" t="s">
+      <c r="A169" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B169" s="1" t="s">
+      <c r="B169" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C169" s="1">
-        <v>16</v>
-      </c>
-      <c r="E169" s="1">
-        <v>0</v>
-      </c>
+      <c r="C169" s="3">
+        <v>17</v>
+      </c>
+      <c r="D169" s="3"/>
+      <c r="E169" s="3">
+        <v>0</v>
+      </c>
+      <c r="F169" s="5"/>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A170" s="3" t="s">
+      <c r="A170" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B170" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C170" s="3">
-        <v>17</v>
-      </c>
-      <c r="D170" s="3"/>
-      <c r="E170" s="3">
-        <v>0</v>
-      </c>
-      <c r="F170" s="5"/>
+      <c r="B170" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C170" s="7">
+        <v>1</v>
+      </c>
+      <c r="D170" s="7"/>
+      <c r="E170" s="7">
+        <v>0</v>
+      </c>
+      <c r="F170" s="8"/>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A171" s="7" t="s">
+      <c r="A171" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B171" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="C171" s="7">
-        <v>1</v>
-      </c>
-      <c r="D171" s="7"/>
-      <c r="E171" s="7">
-        <v>0</v>
-      </c>
-      <c r="F171" s="8"/>
+      <c r="B171" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C171" s="3">
+        <v>1</v>
+      </c>
+      <c r="D171" s="3"/>
+      <c r="E171" s="3">
+        <v>0</v>
+      </c>
+      <c r="F171" s="5"/>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A172" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B172" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C172" s="3">
-        <v>1</v>
-      </c>
-      <c r="D172" s="3"/>
-      <c r="E172" s="3">
-        <v>0</v>
-      </c>
-      <c r="F172" s="5"/>
+      <c r="A172" s="1">
+        <v>3</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C172" s="1">
+        <v>1</v>
+      </c>
+      <c r="D172" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="E172" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
@@ -4180,10 +4180,10 @@
         <v>155</v>
       </c>
       <c r="C173" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D173" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E173" s="1">
         <v>0</v>
@@ -4197,10 +4197,10 @@
         <v>155</v>
       </c>
       <c r="C174" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E174" s="1">
         <v>0</v>
@@ -4214,10 +4214,10 @@
         <v>155</v>
       </c>
       <c r="C175" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E175" s="1">
         <v>0</v>
@@ -4231,10 +4231,10 @@
         <v>155</v>
       </c>
       <c r="C176" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D176" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E176" s="1">
         <v>0</v>
@@ -4248,10 +4248,10 @@
         <v>155</v>
       </c>
       <c r="C177" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D177" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E177" s="1">
         <v>0</v>
@@ -4265,10 +4265,10 @@
         <v>155</v>
       </c>
       <c r="C178" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E178" s="1">
         <v>0</v>
@@ -4282,10 +4282,10 @@
         <v>155</v>
       </c>
       <c r="C179" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E179" s="1">
         <v>0</v>
@@ -4299,10 +4299,10 @@
         <v>155</v>
       </c>
       <c r="C180" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D180" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E180" s="1">
         <v>0</v>
@@ -4316,10 +4316,10 @@
         <v>155</v>
       </c>
       <c r="C181" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E181" s="1">
         <v>0</v>
@@ -4333,10 +4333,10 @@
         <v>155</v>
       </c>
       <c r="C182" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D182" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E182" s="1">
         <v>0</v>
@@ -4350,10 +4350,10 @@
         <v>155</v>
       </c>
       <c r="C183" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D183" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E183" s="1">
         <v>0</v>
@@ -4367,10 +4367,10 @@
         <v>155</v>
       </c>
       <c r="C184" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D184" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E184" s="1">
         <v>0</v>
@@ -4384,13 +4384,16 @@
         <v>155</v>
       </c>
       <c r="C185" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D185" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E185" s="1">
         <v>0</v>
+      </c>
+      <c r="F185" s="4" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
@@ -4401,16 +4404,13 @@
         <v>155</v>
       </c>
       <c r="C186" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D186" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E186" s="1">
         <v>0</v>
-      </c>
-      <c r="F186" s="4" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
@@ -4421,10 +4421,10 @@
         <v>155</v>
       </c>
       <c r="C187" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D187" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E187" s="1">
         <v>0</v>
@@ -4438,10 +4438,10 @@
         <v>155</v>
       </c>
       <c r="C188" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D188" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E188" s="1">
         <v>0</v>
@@ -4455,10 +4455,10 @@
         <v>155</v>
       </c>
       <c r="C189" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D189" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E189" s="1">
         <v>0</v>
@@ -4472,10 +4472,10 @@
         <v>155</v>
       </c>
       <c r="C190" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D190" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E190" s="1">
         <v>0</v>
@@ -4489,10 +4489,10 @@
         <v>155</v>
       </c>
       <c r="C191" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D191" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E191" s="1">
         <v>0</v>
@@ -4506,10 +4506,10 @@
         <v>155</v>
       </c>
       <c r="C192" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D192" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E192" s="1">
         <v>0</v>
@@ -4523,10 +4523,10 @@
         <v>155</v>
       </c>
       <c r="C193" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D193" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E193" s="1">
         <v>0</v>
@@ -4540,10 +4540,10 @@
         <v>155</v>
       </c>
       <c r="C194" s="1">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E194" s="1">
         <v>0</v>
@@ -4557,10 +4557,10 @@
         <v>155</v>
       </c>
       <c r="C195" s="1">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D195" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E195" s="1">
         <v>0</v>
@@ -4574,10 +4574,10 @@
         <v>155</v>
       </c>
       <c r="C196" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D196" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E196" s="1">
         <v>0</v>
@@ -4591,10 +4591,10 @@
         <v>155</v>
       </c>
       <c r="C197" s="1">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D197" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E197" s="1">
         <v>0</v>
@@ -4608,10 +4608,10 @@
         <v>155</v>
       </c>
       <c r="C198" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D198" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E198" s="1">
         <v>0</v>
@@ -4625,10 +4625,10 @@
         <v>155</v>
       </c>
       <c r="C199" s="1">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D199" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E199" s="1">
         <v>0</v>
@@ -4642,10 +4642,10 @@
         <v>155</v>
       </c>
       <c r="C200" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D200" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E200" s="1">
         <v>0</v>
@@ -4659,10 +4659,10 @@
         <v>155</v>
       </c>
       <c r="C201" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D201" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E201" s="1">
         <v>0</v>
@@ -4675,50 +4675,47 @@
       <c r="B202" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C202" s="1">
-        <v>30</v>
+      <c r="C202" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="D202" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E202" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A203" s="1">
+      <c r="A203" s="3">
         <v>3</v>
       </c>
-      <c r="B203" s="1" t="s">
+      <c r="B203" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C203" s="1" t="s">
+      <c r="C203" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D203" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="E203" s="1">
-        <v>0</v>
-      </c>
+      <c r="D203" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="E203" s="3">
+        <v>0</v>
+      </c>
+      <c r="F203" s="5"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A204" s="3">
-        <v>3</v>
-      </c>
-      <c r="B204" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C204" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D204" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E204" s="3">
-        <v>0</v>
-      </c>
-      <c r="F204" s="5"/>
+      <c r="A204" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C204" s="1">
+        <v>1</v>
+      </c>
+      <c r="E204" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
@@ -4728,7 +4725,7 @@
         <v>79</v>
       </c>
       <c r="C205" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E205" s="1">
         <v>0</v>
@@ -4742,7 +4739,7 @@
         <v>79</v>
       </c>
       <c r="C206" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E206" s="1">
         <v>0</v>
@@ -4756,7 +4753,7 @@
         <v>79</v>
       </c>
       <c r="C207" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E207" s="1">
         <v>0</v>
@@ -4770,7 +4767,7 @@
         <v>79</v>
       </c>
       <c r="C208" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E208" s="1">
         <v>0</v>
@@ -4784,7 +4781,7 @@
         <v>79</v>
       </c>
       <c r="C209" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E209" s="1">
         <v>0</v>
@@ -4798,41 +4795,41 @@
         <v>79</v>
       </c>
       <c r="C210" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E210" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A211" s="1" t="s">
+      <c r="A211" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B211" s="1" t="s">
+      <c r="B211" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C211" s="1">
-        <v>7</v>
-      </c>
-      <c r="E211" s="1">
-        <v>0</v>
-      </c>
+      <c r="C211" s="3">
+        <v>8</v>
+      </c>
+      <c r="D211" s="3"/>
+      <c r="E211" s="3">
+        <v>0</v>
+      </c>
+      <c r="F211" s="5"/>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A212" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B212" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C212" s="3">
-        <v>8</v>
-      </c>
-      <c r="D212" s="3"/>
-      <c r="E212" s="3">
-        <v>0</v>
-      </c>
-      <c r="F212" s="5"/>
+      <c r="A212" s="1">
+        <v>4</v>
+      </c>
+      <c r="B212" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C212" s="1">
+        <v>1</v>
+      </c>
+      <c r="E212" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
@@ -4842,7 +4839,7 @@
         <v>157</v>
       </c>
       <c r="C213" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E213" s="1">
         <v>0</v>
@@ -4856,7 +4853,7 @@
         <v>157</v>
       </c>
       <c r="C214" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E214" s="1">
         <v>0</v>
@@ -4870,7 +4867,7 @@
         <v>157</v>
       </c>
       <c r="C215" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E215" s="1">
         <v>0</v>
@@ -4884,7 +4881,7 @@
         <v>157</v>
       </c>
       <c r="C216" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E216" s="1">
         <v>0</v>
@@ -4898,7 +4895,7 @@
         <v>157</v>
       </c>
       <c r="C217" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E217" s="1">
         <v>0</v>
@@ -4912,7 +4909,7 @@
         <v>157</v>
       </c>
       <c r="C218" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E218" s="1">
         <v>0</v>
@@ -4926,7 +4923,7 @@
         <v>157</v>
       </c>
       <c r="C219" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E219" s="1">
         <v>0</v>
@@ -4940,7 +4937,7 @@
         <v>157</v>
       </c>
       <c r="C220" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E220" s="1">
         <v>0</v>
@@ -4954,7 +4951,7 @@
         <v>157</v>
       </c>
       <c r="C221" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E221" s="1">
         <v>0</v>
@@ -4968,7 +4965,7 @@
         <v>157</v>
       </c>
       <c r="C222" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E222" s="1">
         <v>0</v>
@@ -4982,7 +4979,7 @@
         <v>157</v>
       </c>
       <c r="C223" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E223" s="1">
         <v>0</v>
@@ -4996,7 +4993,7 @@
         <v>157</v>
       </c>
       <c r="C224" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E224" s="1">
         <v>0</v>
@@ -5010,7 +5007,7 @@
         <v>157</v>
       </c>
       <c r="C225" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E225" s="1">
         <v>0</v>
@@ -5024,7 +5021,7 @@
         <v>157</v>
       </c>
       <c r="C226" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E226" s="1">
         <v>0</v>
@@ -5038,41 +5035,41 @@
         <v>157</v>
       </c>
       <c r="C227" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E227" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A228" s="1">
+      <c r="A228" s="3">
         <v>4</v>
       </c>
-      <c r="B228" s="1" t="s">
+      <c r="B228" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C228" s="1">
-        <v>16</v>
-      </c>
-      <c r="E228" s="1">
-        <v>0</v>
-      </c>
+      <c r="C228" s="3">
+        <v>17</v>
+      </c>
+      <c r="D228" s="3"/>
+      <c r="E228" s="3">
+        <v>0</v>
+      </c>
+      <c r="F228" s="5"/>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A229" s="3">
-        <v>4</v>
-      </c>
-      <c r="B229" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C229" s="3">
-        <v>17</v>
-      </c>
-      <c r="D229" s="3"/>
-      <c r="E229" s="3">
-        <v>0</v>
-      </c>
-      <c r="F229" s="5"/>
+      <c r="A229" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C229" s="1">
+        <v>1</v>
+      </c>
+      <c r="E229" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
@@ -5082,7 +5079,7 @@
         <v>79</v>
       </c>
       <c r="C230" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E230" s="1">
         <v>0</v>
@@ -5096,7 +5093,7 @@
         <v>79</v>
       </c>
       <c r="C231" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E231" s="1">
         <v>0</v>
@@ -5110,7 +5107,7 @@
         <v>79</v>
       </c>
       <c r="C232" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E232" s="1">
         <v>0</v>
@@ -5124,7 +5121,7 @@
         <v>79</v>
       </c>
       <c r="C233" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E233" s="1">
         <v>0</v>
@@ -5138,7 +5135,7 @@
         <v>79</v>
       </c>
       <c r="C234" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E234" s="1">
         <v>0</v>
@@ -5152,7 +5149,7 @@
         <v>79</v>
       </c>
       <c r="C235" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E235" s="1">
         <v>0</v>
@@ -5166,41 +5163,41 @@
         <v>79</v>
       </c>
       <c r="C236" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E236" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A237" s="1" t="s">
+      <c r="A237" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B237" s="1" t="s">
+      <c r="B237" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C237" s="1">
-        <v>8</v>
-      </c>
-      <c r="E237" s="1">
-        <v>0</v>
-      </c>
+      <c r="C237" s="3">
+        <v>9</v>
+      </c>
+      <c r="D237" s="3"/>
+      <c r="E237" s="3">
+        <v>0</v>
+      </c>
+      <c r="F237" s="5"/>
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A238" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B238" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C238" s="3">
-        <v>9</v>
-      </c>
-      <c r="D238" s="3"/>
-      <c r="E238" s="3">
-        <v>0</v>
-      </c>
-      <c r="F238" s="5"/>
+      <c r="A238" s="1">
+        <v>5</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C238" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E238" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
@@ -5210,7 +5207,7 @@
         <v>159</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E239" s="1">
         <v>0</v>
@@ -5224,7 +5221,7 @@
         <v>159</v>
       </c>
       <c r="C240" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E240" s="1">
         <v>0</v>
@@ -5238,7 +5235,7 @@
         <v>159</v>
       </c>
       <c r="C241" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E241" s="1">
         <v>0</v>
@@ -5252,7 +5249,7 @@
         <v>159</v>
       </c>
       <c r="C242" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E242" s="1">
         <v>0</v>
@@ -5266,7 +5263,7 @@
         <v>159</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E243" s="1">
         <v>0</v>
@@ -5280,7 +5277,7 @@
         <v>159</v>
       </c>
       <c r="C244" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E244" s="1">
         <v>0</v>
@@ -5294,7 +5291,7 @@
         <v>159</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E245" s="1">
         <v>0</v>
@@ -5308,7 +5305,7 @@
         <v>159</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="E246" s="1">
         <v>0</v>
@@ -5322,7 +5319,7 @@
         <v>159</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E247" s="1">
         <v>0</v>
@@ -5336,41 +5333,41 @@
         <v>159</v>
       </c>
       <c r="C248" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E248" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A249" s="1">
+      <c r="A249" s="3">
         <v>5</v>
       </c>
-      <c r="B249" s="1" t="s">
+      <c r="B249" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C249" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E249" s="1">
-        <v>0</v>
-      </c>
+      <c r="C249" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D249" s="3"/>
+      <c r="E249" s="3">
+        <v>0</v>
+      </c>
+      <c r="F249" s="5"/>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A250" s="3">
+      <c r="A250" s="1">
         <v>5</v>
       </c>
-      <c r="B250" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C250" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D250" s="3"/>
-      <c r="E250" s="3">
-        <v>0</v>
-      </c>
-      <c r="F250" s="5"/>
+      <c r="B250" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C250" s="1">
+        <v>1</v>
+      </c>
+      <c r="E250" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
@@ -5380,7 +5377,7 @@
         <v>160</v>
       </c>
       <c r="C251" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E251" s="1">
         <v>0</v>
@@ -5394,7 +5391,7 @@
         <v>160</v>
       </c>
       <c r="C252" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E252" s="1">
         <v>0</v>
@@ -5408,7 +5405,7 @@
         <v>160</v>
       </c>
       <c r="C253" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E253" s="1">
         <v>0</v>
@@ -5422,7 +5419,7 @@
         <v>160</v>
       </c>
       <c r="C254" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E254" s="1">
         <v>0</v>
@@ -5436,7 +5433,7 @@
         <v>160</v>
       </c>
       <c r="C255" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E255" s="1">
         <v>0</v>
@@ -5450,7 +5447,7 @@
         <v>160</v>
       </c>
       <c r="C256" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E256" s="1">
         <v>0</v>
@@ -5464,7 +5461,7 @@
         <v>160</v>
       </c>
       <c r="C257" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E257" s="1">
         <v>0</v>
@@ -5478,7 +5475,7 @@
         <v>160</v>
       </c>
       <c r="C258" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E258" s="1">
         <v>0</v>
@@ -5492,7 +5489,7 @@
         <v>160</v>
       </c>
       <c r="C259" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E259" s="1">
         <v>0</v>
@@ -5506,7 +5503,7 @@
         <v>160</v>
       </c>
       <c r="C260" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E260" s="1">
         <v>0</v>
@@ -5520,41 +5517,41 @@
         <v>160</v>
       </c>
       <c r="C261" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E261" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A262" s="1">
+      <c r="A262" s="3">
         <v>5</v>
       </c>
-      <c r="B262" s="1" t="s">
+      <c r="B262" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C262" s="1">
-        <v>12</v>
-      </c>
-      <c r="E262" s="1">
-        <v>0</v>
-      </c>
+      <c r="C262" s="3">
+        <v>13</v>
+      </c>
+      <c r="D262" s="3"/>
+      <c r="E262" s="3">
+        <v>0</v>
+      </c>
+      <c r="F262" s="5"/>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A263" s="3">
+      <c r="A263" s="1">
         <v>5</v>
       </c>
-      <c r="B263" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C263" s="3">
-        <v>13</v>
-      </c>
-      <c r="D263" s="3"/>
-      <c r="E263" s="3">
-        <v>0</v>
-      </c>
-      <c r="F263" s="5"/>
+      <c r="B263" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C263" s="1">
+        <v>1</v>
+      </c>
+      <c r="E263" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
@@ -5564,7 +5561,7 @@
         <v>161</v>
       </c>
       <c r="C264" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E264" s="1">
         <v>0</v>
@@ -5578,57 +5575,57 @@
         <v>161</v>
       </c>
       <c r="C265" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E265" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A266" s="1">
+      <c r="A266" s="3">
         <v>5</v>
       </c>
-      <c r="B266" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C266" s="1">
-        <v>3</v>
-      </c>
-      <c r="E266" s="1">
-        <v>0</v>
-      </c>
+      <c r="B266" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C266" s="3">
+        <v>1</v>
+      </c>
+      <c r="D266" s="3"/>
+      <c r="E266" s="3">
+        <v>0</v>
+      </c>
+      <c r="F266" s="5"/>
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A267" s="3">
-        <v>5</v>
-      </c>
-      <c r="B267" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C267" s="3">
-        <v>1</v>
-      </c>
-      <c r="D267" s="3"/>
-      <c r="E267" s="3">
-        <v>0</v>
-      </c>
-      <c r="F267" s="5"/>
+      <c r="A267" s="7">
+        <v>6</v>
+      </c>
+      <c r="B267" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C267" s="7">
+        <v>1</v>
+      </c>
+      <c r="D267" s="7"/>
+      <c r="E267" s="7">
+        <v>0</v>
+      </c>
+      <c r="F267" s="8"/>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A268" s="7">
-        <v>6</v>
-      </c>
-      <c r="B268" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="C268" s="7">
-        <v>1</v>
-      </c>
-      <c r="D268" s="7"/>
-      <c r="E268" s="7">
-        <v>0</v>
-      </c>
-      <c r="F268" s="8"/>
+      <c r="A268" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C268" s="1">
+        <v>1</v>
+      </c>
+      <c r="E268" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
@@ -5638,7 +5635,7 @@
         <v>165</v>
       </c>
       <c r="C269" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E269" s="1">
         <v>0</v>
@@ -5652,7 +5649,7 @@
         <v>165</v>
       </c>
       <c r="C270" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E270" s="1">
         <v>0</v>
@@ -5666,7 +5663,7 @@
         <v>165</v>
       </c>
       <c r="C271" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E271" s="1">
         <v>0</v>
@@ -5680,41 +5677,41 @@
         <v>165</v>
       </c>
       <c r="C272" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E272" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A273" s="1" t="s">
+      <c r="A273" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B273" s="1" t="s">
+      <c r="B273" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C273" s="1">
-        <v>5</v>
-      </c>
-      <c r="E273" s="1">
-        <v>0</v>
-      </c>
+      <c r="C273" s="7">
+        <v>6</v>
+      </c>
+      <c r="D273" s="7"/>
+      <c r="E273" s="7">
+        <v>0</v>
+      </c>
+      <c r="F273" s="8"/>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A274" s="7" t="s">
+      <c r="A274" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B274" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="C274" s="7">
-        <v>6</v>
-      </c>
-      <c r="D274" s="7"/>
-      <c r="E274" s="7">
-        <v>0</v>
-      </c>
-      <c r="F274" s="8"/>
+      <c r="B274" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C274" s="1">
+        <v>1</v>
+      </c>
+      <c r="E274" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
@@ -5724,7 +5721,7 @@
         <v>166</v>
       </c>
       <c r="C275" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E275" s="1">
         <v>0</v>
@@ -5738,7 +5735,7 @@
         <v>166</v>
       </c>
       <c r="C276" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E276" s="1">
         <v>0</v>
@@ -5752,44 +5749,30 @@
         <v>166</v>
       </c>
       <c r="C277" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E277" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A278" s="1" t="s">
+      <c r="A278" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B278" s="1" t="s">
+      <c r="B278" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C278" s="1">
-        <v>4</v>
-      </c>
-      <c r="E278" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A279" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B279" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C279" s="3">
+      <c r="C278" s="3">
         <v>5</v>
       </c>
-      <c r="D279" s="3"/>
-      <c r="E279" s="3">
-        <v>0</v>
-      </c>
-      <c r="F279" s="5"/>
+      <c r="D278" s="3"/>
+      <c r="E278" s="3">
+        <v>0</v>
+      </c>
+      <c r="F278" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F279" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}"/>
+  <autoFilter ref="A1:F278" xr:uid="{38511E32-3E3E-40A9-82C1-AB31C8631409}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="iconSet" priority="1">

</xml_diff>